<commit_message>
Fix Crew Payroll row-9 GROSS formula outlier and missing row-54 item number
Row 9's AT (GROSS) formula was =Wages+Corporate+FUI (3 terms), while every
other data row (10-54) uses =Wages+Corporate+FICA+Medi+FUI (5 terms) --
row 9 was a leftover outlier from an earlier edit. Also row 54's ITEM #
(col B) was blank where every other row (1-45) is numbered. Found while
mapping the per-row formula pattern for an upcoming row-growth feature.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/assets/workbooks/texas.xlsx
+++ b/source/assets/workbooks/texas.xlsx
@@ -13626,7 +13626,7 @@
       <c r="AR9" s="382" t="n"/>
       <c r="AS9" s="370" t="n"/>
       <c r="AT9" s="469">
-        <f>N9+O9+R9</f>
+        <f>N9+O9+P9+Q9+R9</f>
         <v/>
       </c>
       <c r="AU9" s="469">
@@ -17367,7 +17367,9 @@
     </row>
     <row r="54">
       <c r="A54" s="456" t="n"/>
-      <c r="B54" s="11" t="n"/>
+      <c r="B54" s="11" t="n">
+        <v>46</v>
+      </c>
       <c r="C54" s="11" t="n"/>
       <c r="D54" s="11" t="n"/>
       <c r="E54" s="287" t="n"/>
@@ -21220,7 +21222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AP264"/>
+  <dimension ref="A1:AP70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="7.28515625" customWidth="1" style="358" min="1" max="1"/>
@@ -24801,207 +24803,12 @@
         <v/>
       </c>
     </row>
-    <row r="69"/>
     <row r="70">
       <c r="I70" s="458">
         <f>I68-I52-I54-I55-I56-I58</f>
         <v/>
       </c>
     </row>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
   </sheetData>
   <autoFilter ref="B8:AG41"/>
   <mergeCells count="6">
@@ -30114,4 +29921,231 @@
   <pageMargins left="0.45" right="0.45" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="20" fitToHeight="0"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100504A511723502843AC0584E68EC60535" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fbd80a4f17478eeb58df59f7f6ca8f1e">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4e7d37e-1dcc-4436-a729-076bff741eab" xmlns:ns3="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="88c3fc8cee6a1370bae988e1d6c9e850" ns2:_="" ns3:_="">
+    <xsd:import namespace="f4e7d37e-1dcc-4436-a729-076bff741eab"/>
+    <xsd:import namespace="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f4e7d37e-1dcc-4436-a729-076bff741eab" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="9be8b6ea-d13c-4d71-97d6-b0474eec2ace" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="18" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{4e8a67d3-72a2-4d67-a918-656f717b250f}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4e7d37e-1dcc-4436-a729-076bff741eab">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="7ff3518b-2e3d-4dfb-a834-48e552d5b5bf" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8C149EF-4D58-42FA-A514-F3E2FCF18756}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AABC933-89DB-42D6-83D5-BA650FDE688C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C701E90E-199F-4E9F-A699-13568B741A66}"/>
 </file>
</xml_diff>